<commit_message>
update: upload latest Case Size.xlsx
</commit_message>
<xml_diff>
--- a/Case Size.xlsx
+++ b/Case Size.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa00\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBA2D4D-71C3-4711-A3B4-48ADEF69E0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4487DCBF-FD93-41C8-8682-90771EABB61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="170">
   <si>
     <t>Category</t>
   </si>
@@ -422,201 +422,209 @@
     </r>
   </si>
   <si>
+    <t>100 GMS</t>
+  </si>
+  <si>
+    <t>48 pack contaning 10 pcs of Cup Dhoop each</t>
+  </si>
+  <si>
+    <t>100 ML Bottle, 72 Bottles in Master Carton</t>
+  </si>
+  <si>
+    <t>1 pack Contain - 10 pcs of Tea light Candles, 12 pcs packed in 1 Outer Carton, 6 Outer Cartons in 1 Master Carton</t>
+  </si>
+  <si>
+    <t>90 gm scented tin smudge candle, wrapped with label sticker. Such 72 pcs packed inside master carton.</t>
+  </si>
+  <si>
+    <t>8 Sticks in a packet,25 packet in a box</t>
+  </si>
+  <si>
+    <t>100 GMS in a packet, 6 packets in a box</t>
+  </si>
+  <si>
+    <t>7 CHAKRA HEXA GIFT PACK</t>
+  </si>
+  <si>
+    <t>7 Packet in an outer packet</t>
+  </si>
+  <si>
+    <t>48 pcs</t>
+  </si>
+  <si>
+    <t>WHITE SAGE CLEANSING COLLECTION GIFT PACK</t>
+  </si>
+  <si>
+    <t>48 sets</t>
+  </si>
+  <si>
+    <t>6 assorated packets in one gift box, such 48 boxes packed inside master carton.</t>
+  </si>
+  <si>
+    <t>YOG CHAKRA GIFT PACK</t>
+  </si>
+  <si>
+    <t>4 Disc in one pack- 2 doz in one inner corrogated box</t>
+  </si>
+  <si>
+    <t>4 Balls in one pack - 2 doz in one inner corrogated box</t>
+  </si>
+  <si>
+    <t>6 Pouches in one pack. 10  sticks in one pouch</t>
+  </si>
+  <si>
+    <t>Paper hexa shape 50grams in a golden pouch with wooden spoon. 12 Hexa Qatari Incense Powder in one Display Box</t>
+  </si>
+  <si>
+    <t>15 gms in one pack, 6 Fragrances  x 2 in one dispenser outer</t>
+  </si>
+  <si>
+    <t>Manifestation candle 125 grms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glass Jar 125 grams Candle </t>
+  </si>
+  <si>
+    <t>10 Sticks in one pack with Crystal and Cards with Affirmation. 1 doz in one Outer</t>
+  </si>
+  <si>
+    <t>15 Grams in a packet,  12 Packs (1 dozen) in a box, 288 Packs (24 dozen) in a master carton</t>
+  </si>
+  <si>
+    <t>Planned to be discontinued</t>
+  </si>
+  <si>
+    <t>ENERGY CLEANSING KIT-  1) Palo Santo Room Spray. - 100ml , 2) Sacred Element - Organic Cones -5- 6 pcs 3) 3) Organic Resins -  10- 15 gsm 4) Organic Herbs -  25-30 gms. 5) Coal Tables for burning - 1 set 6. Terra clay</t>
+  </si>
+  <si>
+    <t>Product - 10 Sticks in a pack, and 12 pack in one dispenser</t>
+  </si>
+  <si>
+    <t>Product - 8 Sticks in a pack, and 12 pack in one dispenser</t>
+  </si>
+  <si>
+    <t>3 sticks in a pack, 6 PACK in one dispenser</t>
+  </si>
+  <si>
+    <t>5 cones in a pack.. 12 pack in one dispenser</t>
+  </si>
+  <si>
+    <t>White Abhir, Gulal, Kumkum, Haldi, Camphor Tablets, Moli, Pooja Supari, Akhata, Agarbatti, Agarbatti Wooden Stand, Janvi Jod, Goddess Photo, Vastra (Pooja Cloth) &amp; Dhoop.</t>
+  </si>
+  <si>
+    <t>Pooja Samagri Kit</t>
+  </si>
+  <si>
+    <t>Aradhana Pooja Oil Pack 900ml</t>
+  </si>
+  <si>
+    <t>1 Bottle x 900 ml, 20Pcs in 1 master carton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aradhana Pooja Oil Pack 450Ml </t>
+  </si>
+  <si>
+    <t>1 Bottle x 450 ml, 40Pcs in 1 master carton</t>
+  </si>
+  <si>
+    <t>HEM Aradhana Camphor - 100g</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Camphor - 100g</t>
+  </si>
+  <si>
+    <t>HEM Aradhana Bhimseni Camphor</t>
+  </si>
+  <si>
+    <t>HEM Aradhana Pure Cow Ghee Diya 100 pcs</t>
+  </si>
+  <si>
+    <t>100 pcs Diya in a box, 4 doz in 1 Master Carton</t>
+  </si>
+  <si>
+    <t>HEM Aradhana Pure Ghee Diya 100 pcs</t>
+  </si>
+  <si>
+    <t>HEM Aradhana Gangajal</t>
+  </si>
+  <si>
+    <t>Gangajal, 24 pc in box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soham Sambrani Cup Dhoop </t>
+  </si>
+  <si>
+    <t>12 pcs in 1 box, 12 dozen in 1 Master Carton</t>
+  </si>
+  <si>
+    <t>Pama Sambrani Cup Dhoop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madhur Guggal Cup Dhhop </t>
+  </si>
+  <si>
+    <t>12 pcs in 1 box, 4 dozen in 1 Master Carton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spell Candle pack of 20 N </t>
+  </si>
+  <si>
+    <t>Votive Shot Glass Candles 40G</t>
+  </si>
+  <si>
+    <t>1 Candle = 40 gms,     48 Pcs (4 Dozen in 1 master carton)</t>
+  </si>
+  <si>
+    <t>7 Chakra  Tea Light Fragrance  Candle</t>
+  </si>
+  <si>
+    <t>GLASS JAR  CANDLE 185 GMS</t>
+  </si>
+  <si>
+    <t>125 gms Scented Candle</t>
+  </si>
+  <si>
+    <t>6 hexa pack in packet</t>
+  </si>
+  <si>
+    <t>7 Diffrenet types of Stones in one pack.,12 packs in 1 Outer Carton,6 Outer Cartons in one Master Carton</t>
+  </si>
+  <si>
+    <t>20 Sticks in a packet, 6 packet in a box, 2 boxes make 1 Dozen, 25 dozen in 1 master carton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 gm in a packet, 12 packet in 1 dozen,,,24 dozen in 1 master carton </t>
+  </si>
+  <si>
+    <t>25 gm in a packet, 12 packets in 1 dozen,24 dozen in master carton</t>
+  </si>
+  <si>
+    <t>20 Sticks in a packet, 6 packet in a box,2 boxes make 1 Dozen, 25 dozen in 1 master carton</t>
+  </si>
+  <si>
+    <t>12 pcs packed inside the display box.,8 display box packed inside master carton</t>
+  </si>
+  <si>
+    <t>Gift Pack Contain single pc of Yog Chakra 100ml room freshener, 15gm Masala incense stick,Yog Chakra cone &amp;Wooden incense holder</t>
+  </si>
+  <si>
+    <t>1 pack Contain -7 pcs of Tea light Candles.,12 pcs packed in 1 Outer Carton.,6 Outer Cartons in 1 Master Carton</t>
+  </si>
+  <si>
+    <t>1 pack Contain - 10 pcs of Tea light Candles.,12 pcs packed in 1 Outer Carton.,6 Outer Cartons in 1 Master Carton</t>
+  </si>
+  <si>
+    <t>20 candles unsencted ,Extended Burn Time: Each 4-inch tall unscented candle burns continuously for up to 2 hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>DHOOP</t>
+  </si>
+  <si>
     <r>
-      <t>DHOOP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF3D2020"/>
-        <rFont val="Aptos Display"/>
-        <scheme val="major"/>
-      </rPr>
-      <t>    25 GMS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>DHOOP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF3D2020"/>
-        <rFont val="Aptos Display"/>
-        <scheme val="major"/>
-      </rPr>
-      <t>   60 GRMS</t>
-    </r>
-  </si>
-  <si>
-    <t>25 GMS in a packet,12 packet in a box</t>
-  </si>
-  <si>
-    <t>100 GMS</t>
-  </si>
-  <si>
-    <t>48 pack contaning 10 pcs of Cup Dhoop each</t>
-  </si>
-  <si>
-    <t>100 ML Bottle, 72 Bottles in Master Carton</t>
-  </si>
-  <si>
-    <t>1 pack Contain - 10 pcs of Tea light Candles, 12 pcs packed in 1 Outer Carton, 6 Outer Cartons in 1 Master Carton</t>
-  </si>
-  <si>
-    <t>90 gm scented tin smudge candle, wrapped with label sticker. Such 72 pcs packed inside master carton.</t>
-  </si>
-  <si>
-    <t>8 Sticks in a packet,25 packet in a box</t>
-  </si>
-  <si>
-    <t>100 GMS in a packet, 6 packets in a box</t>
-  </si>
-  <si>
-    <t>7 CHAKRA HEXA GIFT PACK</t>
-  </si>
-  <si>
-    <t>7 Packet in an outer packet</t>
-  </si>
-  <si>
-    <t>48 pcs</t>
-  </si>
-  <si>
-    <t>WHITE SAGE CLEANSING COLLECTION GIFT PACK</t>
-  </si>
-  <si>
-    <t>48 sets</t>
-  </si>
-  <si>
-    <t>6 assorated packets in one gift box, such 48 boxes packed inside master carton.</t>
-  </si>
-  <si>
-    <t>YOG CHAKRA GIFT PACK</t>
-  </si>
-  <si>
-    <t>4 Disc in one pack- 2 doz in one inner corrogated box</t>
-  </si>
-  <si>
-    <t>4 Balls in one pack - 2 doz in one inner corrogated box</t>
-  </si>
-  <si>
-    <t>6 Pouches in one pack. 10  sticks in one pouch</t>
-  </si>
-  <si>
-    <t>Paper hexa shape 50grams in a golden pouch with wooden spoon. 12 Hexa Qatari Incense Powder in one Display Box</t>
-  </si>
-  <si>
-    <t>15 gms in one pack, 6 Fragrances  x 2 in one dispenser outer</t>
-  </si>
-  <si>
-    <t>Manifestation candle 125 grms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glass Jar 125 grams Candle </t>
-  </si>
-  <si>
-    <t>10 Sticks in one pack with Crystal and Cards with Affirmation. 1 doz in one Outer</t>
-  </si>
-  <si>
-    <t>15 Grams in a packet,  12 Packs (1 dozen) in a box, 288 Packs (24 dozen) in a master carton</t>
-  </si>
-  <si>
-    <t>Planned to be discontinued</t>
-  </si>
-  <si>
-    <t>ENERGY CLEANSING KIT-  1) Palo Santo Room Spray. - 100ml , 2) Sacred Element - Organic Cones -5- 6 pcs 3) 3) Organic Resins -  10- 15 gsm 4) Organic Herbs -  25-30 gms. 5) Coal Tables for burning - 1 set 6. Terra clay</t>
-  </si>
-  <si>
-    <t>Product - 10 Sticks in a pack, and 12 pack in one dispenser</t>
-  </si>
-  <si>
-    <t>Product - 8 Sticks in a pack, and 12 pack in one dispenser</t>
-  </si>
-  <si>
-    <t>3 sticks in a pack, 6 PACK in one dispenser</t>
-  </si>
-  <si>
-    <t>5 cones in a pack.. 12 pack in one dispenser</t>
-  </si>
-  <si>
-    <t>White Abhir, Gulal, Kumkum, Haldi, Camphor Tablets, Moli, Pooja Supari, Akhata, Agarbatti, Agarbatti Wooden Stand, Janvi Jod, Goddess Photo, Vastra (Pooja Cloth) &amp; Dhoop.</t>
-  </si>
-  <si>
-    <t>Pooja Samagri Kit</t>
-  </si>
-  <si>
-    <t>Aradhana Pooja Oil Pack 900ml</t>
-  </si>
-  <si>
-    <t>1 Bottle x 900 ml, 20Pcs in 1 master carton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aradhana Pooja Oil Pack 450Ml </t>
-  </si>
-  <si>
-    <t>1 Bottle x 450 ml, 40Pcs in 1 master carton</t>
-  </si>
-  <si>
-    <t>HEM Aradhana Camphor - 100g</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Camphor - 100g</t>
-  </si>
-  <si>
-    <t>HEM Aradhana Bhimseni Camphor</t>
-  </si>
-  <si>
-    <t>HEM Aradhana Pure Cow Ghee Diya 100 pcs</t>
-  </si>
-  <si>
-    <t>100 pcs Diya in a box, 4 doz in 1 Master Carton</t>
-  </si>
-  <si>
-    <t>HEM Aradhana Pure Ghee Diya 100 pcs</t>
-  </si>
-  <si>
-    <t>HEM Aradhana Gangajal</t>
-  </si>
-  <si>
-    <t>Gangajal, 24 pc in box</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soham Sambrani Cup Dhoop </t>
-  </si>
-  <si>
-    <t>12 pcs in 1 box, 12 dozen in 1 Master Carton</t>
-  </si>
-  <si>
-    <t>Pama Sambrani Cup Dhoop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Madhur Guggal Cup Dhhop </t>
-  </si>
-  <si>
-    <t>12 pcs in 1 box, 4 dozen in 1 Master Carton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spell Candle pack of 20 N </t>
-  </si>
-  <si>
-    <t>Votive Shot Glass Candles 40G</t>
-  </si>
-  <si>
-    <t>1 Candle = 40 gms,     48 Pcs (4 Dozen in 1 master carton)</t>
-  </si>
-  <si>
-    <t>7 Chakra  Tea Light Fragrance  Candle</t>
-  </si>
-  <si>
-    <t>GLASS JAR  CANDLE 185 GMS</t>
-  </si>
-  <si>
-    <t>125 gms Scented Candle</t>
-  </si>
-  <si>
-    <r>
-      <t>Regular CONE</t>
+      <t>CONE</t>
     </r>
     <r>
       <rPr>
@@ -627,39 +635,6 @@
       </rPr>
       <t> </t>
     </r>
-  </si>
-  <si>
-    <t>6 hexa pack in packet</t>
-  </si>
-  <si>
-    <t>7 Diffrenet types of Stones in one pack.,12 packs in 1 Outer Carton,6 Outer Cartons in one Master Carton</t>
-  </si>
-  <si>
-    <t>20 Sticks in a packet, 6 packet in a box, 2 boxes make 1 Dozen, 25 dozen in 1 master carton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 gm in a packet, 12 packet in 1 dozen,,,24 dozen in 1 master carton </t>
-  </si>
-  <si>
-    <t>25 gm in a packet, 12 packets in 1 dozen,24 dozen in master carton</t>
-  </si>
-  <si>
-    <t>20 Sticks in a packet, 6 packet in a box,2 boxes make 1 Dozen, 25 dozen in 1 master carton</t>
-  </si>
-  <si>
-    <t>12 pcs packed inside the display box.,8 display box packed inside master carton</t>
-  </si>
-  <si>
-    <t>Gift Pack Contain single pc of Yog Chakra 100ml room freshener, 15gm Masala incense stick,Yog Chakra cone &amp;Wooden incense holder</t>
-  </si>
-  <si>
-    <t>1 pack Contain -7 pcs of Tea light Candles.,12 pcs packed in 1 Outer Carton.,6 Outer Cartons in 1 Master Carton</t>
-  </si>
-  <si>
-    <t>1 pack Contain - 10 pcs of Tea light Candles.,12 pcs packed in 1 Outer Carton.,6 Outer Cartons in 1 Master Carton</t>
-  </si>
-  <si>
-    <t>20 candles unsencted ,Extended Burn Time: Each 4-inch tall unscented candle burns continuously for up to 2 hours.</t>
   </si>
 </sst>
 </file>
@@ -9738,7 +9713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="69.1796875" style="4" customWidth="1"/>
@@ -9749,7 +9724,7 @@
     <col min="6" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.6328125" style="5" customWidth="1"/>
     <col min="10" max="10" width="19.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9764,7 +9739,9 @@
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
-      <c r="I1" s="11"/>
+      <c r="I1" s="11" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="28" t="s">
@@ -9800,7 +9777,7 @@
         <v>45</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>18</v>
@@ -9829,7 +9806,7 @@
         <v>45</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>19</v>
@@ -9858,7 +9835,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>11</v>
@@ -9887,7 +9864,7 @@
         <v>45</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>9</v>
@@ -10151,7 +10128,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>18</v>
@@ -10180,7 +10157,7 @@
         <v>83</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>40</v>
@@ -10297,7 +10274,7 @@
         <v>80</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>22</v>
@@ -10354,7 +10331,7 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="29" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>95</v>
@@ -10384,7 +10361,7 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="30" t="s">
-        <v>103</v>
+        <v>168</v>
       </c>
       <c r="B23" s="24" t="s">
         <v>98</v>
@@ -10414,139 +10391,152 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="30" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="16"/>
+        <v>25</v>
+      </c>
+      <c r="D24" s="10">
+        <v>27</v>
+      </c>
+      <c r="E24" s="10">
+        <v>25.3</v>
+      </c>
+      <c r="F24" s="10">
+        <v>61.5</v>
+      </c>
+      <c r="G24" s="10">
+        <v>46</v>
+      </c>
+      <c r="H24" s="10">
+        <v>35</v>
+      </c>
+      <c r="I24" s="16">
+        <v>9.9015000000000006E-2</v>
+      </c>
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:12">
-      <c r="A25" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>99</v>
+      <c r="A25" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>97</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D25" s="10">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E25" s="10">
-        <v>25.3</v>
+        <v>19</v>
       </c>
       <c r="F25" s="10">
-        <v>61.5</v>
+        <v>42.5</v>
       </c>
       <c r="G25" s="10">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="H25" s="10">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="I25" s="16">
-        <v>9.9015000000000006E-2</v>
+        <v>6.6640000000000005E-2</v>
       </c>
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D26" s="10">
-        <v>20</v>
+        <v>12.75</v>
       </c>
       <c r="E26" s="10">
-        <v>19</v>
+        <v>11.2</v>
       </c>
       <c r="F26" s="10">
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="G26" s="10">
-        <v>32</v>
+        <v>28.2</v>
       </c>
       <c r="H26" s="10">
-        <v>49</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I26" s="16">
-        <v>6.6640000000000005E-2</v>
+        <v>3.6801E-2</v>
       </c>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" ht="15" thickBot="1">
       <c r="A27" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>100</v>
+        <v>156</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D27" s="10">
-        <v>12.75</v>
+        <v>13.8</v>
       </c>
       <c r="E27" s="10">
-        <v>11.2</v>
+        <v>12.8</v>
       </c>
       <c r="F27" s="10">
-        <v>37.5</v>
+        <v>58.5</v>
       </c>
       <c r="G27" s="10">
-        <v>28.2</v>
+        <v>31</v>
       </c>
       <c r="H27" s="10">
-        <v>34.799999999999997</v>
+        <v>51.2</v>
       </c>
       <c r="I27" s="16">
-        <v>3.6801E-2</v>
+        <v>9.2851200000000009E-2</v>
       </c>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:12" ht="15" thickBot="1">
-      <c r="A28" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>160</v>
+      <c r="A28" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>110</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>15</v>
+        <v>111</v>
       </c>
       <c r="D28" s="10">
-        <v>13.8</v>
+        <v>16.3</v>
       </c>
       <c r="E28" s="10">
-        <v>12.8</v>
+        <v>15.1</v>
       </c>
       <c r="F28" s="10">
-        <v>58.5</v>
+        <v>42</v>
       </c>
       <c r="G28" s="10">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="H28" s="10">
-        <v>51.2</v>
+        <v>53</v>
       </c>
       <c r="I28" s="16">
-        <v>9.2851200000000009E-2</v>
+        <f t="shared" ref="I28" si="0">+F28*G28*H28/1000000</f>
+        <v>8.0135999999999999E-2</v>
       </c>
       <c r="J28" s="2"/>
     </row>
@@ -10554,386 +10544,367 @@
       <c r="A29" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>114</v>
-      </c>
       <c r="D29" s="10">
-        <v>16.3</v>
+        <v>15.3</v>
       </c>
       <c r="E29" s="10">
-        <v>15.1</v>
+        <v>14.3</v>
       </c>
       <c r="F29" s="10">
-        <v>42</v>
+        <v>42.5</v>
       </c>
       <c r="G29" s="10">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H29" s="10">
-        <v>53</v>
+        <v>54.5</v>
       </c>
       <c r="I29" s="16">
-        <f t="shared" ref="I29" si="0">+F29*G29*H29/1000000</f>
-        <v>8.0135999999999999E-2</v>
+        <v>9.2766407999999995E-2</v>
       </c>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:12" ht="15" thickBot="1">
+    <row r="30" spans="1:12" ht="29.5" thickBot="1">
       <c r="A30" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="B30" s="18" t="s">
-        <v>117</v>
+      <c r="B30" s="19" t="s">
+        <v>163</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="D30" s="10">
-        <v>15.3</v>
+        <v>11.5</v>
       </c>
       <c r="E30" s="10">
-        <v>14.3</v>
+        <v>10.9</v>
       </c>
       <c r="F30" s="10">
-        <v>42.5</v>
+        <v>46</v>
       </c>
       <c r="G30" s="10">
-        <v>40</v>
+        <v>40.5</v>
       </c>
       <c r="H30" s="10">
-        <v>54.5</v>
+        <v>47</v>
       </c>
       <c r="I30" s="16">
-        <v>9.2766407999999995E-2</v>
+        <f>F30*G30*H30/1000000</f>
+        <v>8.7561E-2</v>
       </c>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:12" ht="29.5" thickBot="1">
-      <c r="A31" s="31" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>167</v>
+    <row r="31" spans="1:12">
+      <c r="A31" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>95</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D31" s="10">
-        <v>11.5</v>
+        <v>13.5</v>
       </c>
       <c r="E31" s="10">
-        <v>10.9</v>
+        <v>12.4</v>
       </c>
       <c r="F31" s="10">
-        <v>46</v>
+        <v>47.5</v>
       </c>
       <c r="G31" s="10">
-        <v>40.5</v>
+        <v>44.3</v>
       </c>
       <c r="H31" s="10">
-        <v>47</v>
+        <v>32.5</v>
       </c>
       <c r="I31" s="16">
-        <f>F31*G31*H31/1000000</f>
-        <v>8.7561E-2</v>
-      </c>
-      <c r="J31" s="2"/>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>95</v>
+        <v>160</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="D32" s="10">
-        <v>13.5</v>
+        <v>15.3</v>
       </c>
       <c r="E32" s="10">
-        <v>12.4</v>
-      </c>
-      <c r="F32" s="10">
-        <v>47.5</v>
-      </c>
-      <c r="G32" s="10">
-        <v>44.3</v>
-      </c>
-      <c r="H32" s="10">
-        <v>32.5</v>
-      </c>
-      <c r="I32" s="16">
-        <v>7.0000000000000007E-2</v>
-      </c>
+        <v>13.95</v>
+      </c>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="16"/>
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D33" s="10">
-        <v>15.3</v>
+        <v>11</v>
       </c>
       <c r="E33" s="10">
-        <v>13.95</v>
-      </c>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="F33" s="10">
+        <v>41.5</v>
+      </c>
+      <c r="G33" s="10">
+        <v>27.5</v>
+      </c>
+      <c r="H33" s="10">
+        <v>21</v>
+      </c>
+      <c r="I33" s="16">
+        <v>2.3966250000000001E-2</v>
+      </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>105</v>
+        <v>35</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>94</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D34" s="10">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E34" s="10">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F34" s="10">
-        <v>41.5</v>
+        <v>63</v>
       </c>
       <c r="G34" s="10">
-        <v>27.5</v>
+        <v>32</v>
       </c>
       <c r="H34" s="10">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="I34" s="16">
-        <v>2.3966250000000001E-2</v>
-      </c>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
+        <v>8.2655999999999993E-2</v>
+      </c>
     </row>
     <row r="35" spans="1:12">
       <c r="A35" s="15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D35" s="10">
-        <v>15</v>
+        <v>10.5</v>
       </c>
       <c r="E35" s="10">
-        <v>14</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="F35" s="10">
-        <v>63</v>
+        <v>37.5</v>
       </c>
       <c r="G35" s="10">
-        <v>32</v>
+        <v>30.5</v>
       </c>
       <c r="H35" s="10">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="I35" s="16">
-        <v>8.2655999999999993E-2</v>
+        <v>5.2999999999999999E-2</v>
       </c>
     </row>
     <row r="36" spans="1:12">
       <c r="A36" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="D36" s="10">
-        <v>10.5</v>
+        <v>10.72</v>
       </c>
       <c r="E36" s="10">
-        <v>9.6999999999999993</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="F36" s="10">
-        <v>37.5</v>
+        <v>28</v>
       </c>
       <c r="G36" s="10">
-        <v>30.5</v>
+        <v>28</v>
       </c>
       <c r="H36" s="10">
-        <v>46</v>
+        <v>34.5</v>
       </c>
       <c r="I36" s="16">
-        <v>5.2999999999999999E-2</v>
+        <v>2.7047999999999999E-2</v>
       </c>
     </row>
     <row r="37" spans="1:12">
       <c r="A37" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D37" s="10">
-        <v>10.72</v>
+        <v>13</v>
       </c>
       <c r="E37" s="10">
-        <v>9.7200000000000006</v>
+        <v>11</v>
       </c>
       <c r="F37" s="10">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="G37" s="10">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H37" s="10">
-        <v>34.5</v>
+        <v>39</v>
       </c>
       <c r="I37" s="16">
-        <v>2.7047999999999999E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="38" spans="1:12">
       <c r="A38" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="D38" s="10">
-        <v>13</v>
+        <v>11.4</v>
       </c>
       <c r="E38" s="10">
         <v>11</v>
       </c>
       <c r="F38" s="10">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="G38" s="10">
-        <v>22</v>
+        <v>28.2</v>
       </c>
       <c r="H38" s="10">
-        <v>39</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I38" s="16">
-        <v>0.03</v>
+        <v>3.6801E-2</v>
       </c>
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D39" s="10">
-        <v>11.4</v>
+        <v>23</v>
       </c>
       <c r="E39" s="10">
-        <v>11</v>
+        <v>21.5</v>
       </c>
       <c r="F39" s="10">
-        <v>37.5</v>
+        <v>41.5</v>
       </c>
       <c r="G39" s="10">
-        <v>28.2</v>
+        <v>41.5</v>
       </c>
       <c r="H39" s="10">
-        <v>34.799999999999997</v>
+        <v>54.7</v>
       </c>
       <c r="I39" s="16">
-        <v>3.6801E-2</v>
+        <v>9.4207075000000001E-2</v>
       </c>
     </row>
     <row r="40" spans="1:12">
       <c r="A40" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="D40" s="10">
+        <v>24</v>
+      </c>
+      <c r="E40" s="10">
         <v>23</v>
       </c>
-      <c r="E40" s="10">
-        <v>21.5</v>
-      </c>
       <c r="F40" s="10">
-        <v>41.5</v>
+        <v>51.5</v>
       </c>
       <c r="G40" s="10">
-        <v>41.5</v>
+        <v>33.5</v>
       </c>
       <c r="H40" s="10">
-        <v>54.7</v>
+        <v>60</v>
       </c>
       <c r="I40" s="16">
-        <v>9.4207075000000001E-2</v>
+        <v>0.104</v>
       </c>
     </row>
     <row r="41" spans="1:12">
-      <c r="A41" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D41" s="10">
-        <v>24</v>
-      </c>
-      <c r="E41" s="10">
-        <v>23</v>
-      </c>
-      <c r="F41" s="10">
-        <v>51.5</v>
-      </c>
-      <c r="G41" s="10">
-        <v>33.5</v>
-      </c>
-      <c r="H41" s="10">
-        <v>60</v>
-      </c>
-      <c r="I41" s="16">
-        <v>0.104</v>
-      </c>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="16"/>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" ht="23">
+      <c r="A42" s="32" t="s">
+        <v>62</v>
+      </c>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
@@ -10942,260 +10913,281 @@
       <c r="H42" s="10"/>
       <c r="I42" s="16"/>
     </row>
-    <row r="43" spans="1:12" ht="23">
-      <c r="A43" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="16"/>
+    <row r="43" spans="1:12">
+      <c r="A43" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I43" s="16" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="44" spans="1:12">
-      <c r="A44" s="33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>1</v>
+      <c r="A44" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>116</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I44" s="16" t="s">
-        <v>7</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10">
+        <v>50.9</v>
+      </c>
+      <c r="G44" s="10">
+        <v>39.6</v>
+      </c>
+      <c r="H44" s="10">
+        <v>60</v>
+      </c>
+      <c r="I44" s="16">
+        <v>0.12093840000000002</v>
+      </c>
+      <c r="J44" s="3"/>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
+      <c r="D45" s="10">
+        <v>27</v>
+      </c>
+      <c r="E45" s="10">
+        <v>24</v>
+      </c>
       <c r="F45" s="10">
-        <v>50.9</v>
+        <v>55</v>
       </c>
       <c r="G45" s="10">
-        <v>39.6</v>
+        <v>33</v>
       </c>
       <c r="H45" s="10">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="I45" s="16">
-        <v>0.12093840000000002</v>
+        <v>0.12705</v>
       </c>
       <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="D46" s="10">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E46" s="10">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F46" s="10">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G46" s="10">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="H46" s="10">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="I46" s="16">
-        <v>0.12705</v>
+        <v>0.11015999999999999</v>
       </c>
       <c r="J46" s="3"/>
     </row>
     <row r="47" spans="1:12">
       <c r="A47" s="15" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="C47" s="10" t="s">
-        <v>63</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="C47" s="10"/>
       <c r="D47" s="10">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E47" s="10">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="F47" s="10">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G47" s="10">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="H47" s="10">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I47" s="16">
-        <v>0.11015999999999999</v>
+        <v>7.0223999999999995E-2</v>
       </c>
       <c r="J47" s="3"/>
     </row>
     <row r="48" spans="1:12">
       <c r="A48" s="15" t="s">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="C48" s="10"/>
+        <v>120</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>19</v>
+      </c>
       <c r="D48" s="10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E48" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" s="10">
-        <v>38</v>
+        <v>46.5</v>
       </c>
       <c r="G48" s="10">
-        <v>56</v>
+        <v>36.5</v>
       </c>
       <c r="H48" s="10">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="I48" s="16">
-        <v>7.0223999999999995E-2</v>
+        <f>(F48*G48*H48)/1000000</f>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J48" s="3"/>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="15" t="s">
-        <v>51</v>
+        <v>121</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="E49" s="10">
-        <v>5</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="F49" s="10">
-        <v>46.5</v>
+        <v>36</v>
       </c>
       <c r="G49" s="10">
-        <v>36.5</v>
+        <v>28</v>
       </c>
       <c r="H49" s="10">
-        <v>55</v>
+        <v>33.5</v>
       </c>
       <c r="I49" s="16">
         <f>(F49*G49*H49)/1000000</f>
-        <v>9.3348749999999994E-2</v>
+        <v>3.3767999999999999E-2</v>
       </c>
       <c r="J49" s="3"/>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="15" t="s">
-        <v>124</v>
+        <v>52</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="D50" s="10">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="E50" s="10">
-        <v>9.3000000000000007</v>
+        <v>5</v>
       </c>
       <c r="F50" s="10">
-        <v>36</v>
+        <v>46.5</v>
       </c>
       <c r="G50" s="10">
-        <v>28</v>
+        <v>36.5</v>
       </c>
       <c r="H50" s="10">
-        <v>33.5</v>
+        <v>55</v>
       </c>
       <c r="I50" s="16">
         <f>(F50*G50*H50)/1000000</f>
-        <v>3.3767999999999999E-2</v>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J50" s="3"/>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="D51" s="10">
-        <v>7</v>
+        <v>10.3</v>
       </c>
       <c r="E51" s="10">
-        <v>5</v>
+        <v>9.6</v>
       </c>
       <c r="F51" s="10">
-        <v>46.5</v>
+        <v>49</v>
       </c>
       <c r="G51" s="10">
-        <v>36.5</v>
+        <v>27</v>
       </c>
       <c r="H51" s="10">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="I51" s="16">
         <f>(F51*G51*H51)/1000000</f>
-        <v>9.3348749999999994E-2</v>
-      </c>
-      <c r="J51" s="3"/>
+        <v>5.9534999999999998E-2</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C52" s="10" t="s">
         <v>11</v>
@@ -11216,138 +11208,135 @@
         <v>45</v>
       </c>
       <c r="I52" s="16">
-        <f>(F52*G52*H52)/1000000</f>
+        <f t="shared" ref="I52" si="1">(F52*G52*H52)/1000000</f>
         <v>5.9534999999999998E-2</v>
       </c>
-      <c r="J52" s="3" t="s">
-        <v>128</v>
-      </c>
+      <c r="J52" s="3"/>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="D53" s="10">
-        <v>10.3</v>
+        <v>10.72</v>
       </c>
       <c r="E53" s="10">
-        <v>9.6</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="F53" s="10">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="G53" s="10">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H53" s="10">
-        <v>45</v>
+        <v>34.5</v>
       </c>
       <c r="I53" s="16">
-        <f t="shared" ref="I53" si="1">(F53*G53*H53)/1000000</f>
-        <v>5.9534999999999998E-2</v>
+        <v>2.7047999999999999E-2</v>
       </c>
       <c r="J53" s="3"/>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D54" s="10">
-        <v>10.72</v>
+        <v>12.75</v>
       </c>
       <c r="E54" s="10">
-        <v>9.7200000000000006</v>
+        <v>11.2</v>
       </c>
       <c r="F54" s="10">
-        <v>28</v>
+        <v>37.5</v>
       </c>
       <c r="G54" s="10">
-        <v>28</v>
+        <v>28.2</v>
       </c>
       <c r="H54" s="10">
-        <v>34.5</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I54" s="16">
-        <v>2.7047999999999999E-2</v>
+        <v>3.6801E-2</v>
       </c>
       <c r="J54" s="3"/>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" ht="29">
       <c r="A55" s="15" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>65</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="C55" s="10"/>
       <c r="D55" s="10">
-        <v>12.75</v>
+        <v>16</v>
       </c>
       <c r="E55" s="10">
-        <v>11.2</v>
+        <v>15</v>
       </c>
       <c r="F55" s="10">
-        <v>37.5</v>
+        <v>22</v>
       </c>
       <c r="G55" s="10">
-        <v>28.2</v>
+        <v>7.8</v>
       </c>
       <c r="H55" s="10">
-        <v>34.799999999999997</v>
+        <v>21</v>
       </c>
       <c r="I55" s="16">
-        <v>3.6801E-2</v>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J55" s="3"/>
     </row>
-    <row r="56" spans="1:10" ht="29">
+    <row r="56" spans="1:10">
       <c r="A56" s="15" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="C56" s="10"/>
+        <v>127</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>32</v>
+      </c>
       <c r="D56" s="10">
-        <v>16</v>
+        <v>10.3</v>
       </c>
       <c r="E56" s="10">
-        <v>15</v>
+        <v>9.6</v>
       </c>
       <c r="F56" s="10">
-        <v>22</v>
+        <v>21.8</v>
       </c>
       <c r="G56" s="10">
-        <v>7.8</v>
+        <v>5.6</v>
       </c>
       <c r="H56" s="10">
-        <v>21</v>
+        <v>14.1</v>
       </c>
       <c r="I56" s="16">
-        <v>9.3348749999999994E-2</v>
+        <v>9.4E-2</v>
       </c>
       <c r="J56" s="3"/>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C57" s="10" t="s">
         <v>32</v>
@@ -11374,129 +11363,108 @@
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D58" s="10">
-        <v>10.3</v>
+        <v>15.6</v>
       </c>
       <c r="E58" s="10">
-        <v>9.6</v>
+        <v>14.6</v>
       </c>
       <c r="F58" s="10">
-        <v>21.8</v>
+        <v>54</v>
       </c>
       <c r="G58" s="10">
-        <v>5.6</v>
+        <v>30</v>
       </c>
       <c r="H58" s="10">
-        <v>14.1</v>
+        <v>44.5</v>
       </c>
       <c r="I58" s="16">
-        <v>9.4E-2</v>
+        <f t="shared" ref="I58:I59" si="2">(F58*G58*H58)/1000000</f>
+        <v>7.2090000000000001E-2</v>
       </c>
       <c r="J58" s="3"/>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="D59" s="10">
-        <v>15.6</v>
+        <v>20</v>
       </c>
       <c r="E59" s="10">
-        <v>14.6</v>
+        <v>19.2</v>
       </c>
       <c r="F59" s="10">
-        <v>54</v>
+        <v>48.5</v>
       </c>
       <c r="G59" s="10">
-        <v>30</v>
+        <v>40.5</v>
       </c>
       <c r="H59" s="10">
-        <v>44.5</v>
+        <v>42</v>
       </c>
       <c r="I59" s="16">
-        <f t="shared" ref="I59:I60" si="2">(F59*G59*H59)/1000000</f>
-        <v>7.2090000000000001E-2</v>
+        <f t="shared" si="2"/>
+        <v>8.2498500000000002E-2</v>
       </c>
       <c r="J59" s="3"/>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D60" s="10">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E60" s="10">
-        <v>19.2</v>
+        <v>28</v>
       </c>
       <c r="F60" s="10">
-        <v>48.5</v>
+        <f>12*4</f>
+        <v>48</v>
       </c>
       <c r="G60" s="10">
-        <v>40.5</v>
+        <f>25.5*2</f>
+        <v>51</v>
       </c>
       <c r="H60" s="10">
-        <v>42</v>
+        <f>2.5*18</f>
+        <v>45</v>
       </c>
       <c r="I60" s="16">
-        <f t="shared" si="2"/>
-        <v>8.2498500000000002E-2</v>
+        <f>(F60*G60*H60)/1000000</f>
+        <v>0.11015999999999999</v>
       </c>
       <c r="J60" s="3"/>
     </row>
     <row r="61" spans="1:10">
-      <c r="A61" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B61" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="C61" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D61" s="10">
-        <v>30</v>
-      </c>
-      <c r="E61" s="10">
-        <v>28</v>
-      </c>
-      <c r="F61" s="10">
-        <f>12*4</f>
-        <v>48</v>
-      </c>
-      <c r="G61" s="10">
-        <f>25.5*2</f>
-        <v>51</v>
-      </c>
-      <c r="H61" s="10">
-        <f>2.5*18</f>
-        <v>45</v>
-      </c>
-      <c r="I61" s="16">
-        <f>(F61*G61*H61)/1000000</f>
-        <v>0.11015999999999999</v>
-      </c>
-      <c r="J61" s="3"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="16"/>
     </row>
     <row r="62" spans="1:10">
       <c r="C62" s="10"/>
@@ -11507,7 +11475,10 @@
       <c r="H62" s="10"/>
       <c r="I62" s="16"/>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" ht="23.5">
+      <c r="A63" s="34" t="s">
+        <v>73</v>
+      </c>
       <c r="C63" s="10"/>
       <c r="D63" s="10"/>
       <c r="E63" s="10"/>
@@ -11516,53 +11487,70 @@
       <c r="H63" s="10"/>
       <c r="I63" s="16"/>
     </row>
-    <row r="64" spans="1:10" ht="23.5">
-      <c r="A64" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="16"/>
+    <row r="64" spans="1:10">
+      <c r="A64" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F64" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H64" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I64" s="16" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="65" spans="1:9">
-      <c r="A65" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>1</v>
+      <c r="A65" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" s="25" t="s">
+        <v>146</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F65" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G65" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I65" s="16" t="s">
-        <v>7</v>
+        <v>71</v>
+      </c>
+      <c r="D65" s="10">
+        <v>25</v>
+      </c>
+      <c r="E65" s="10">
+        <v>24</v>
+      </c>
+      <c r="F65" s="10">
+        <v>58</v>
+      </c>
+      <c r="G65" s="10">
+        <v>43.5</v>
+      </c>
+      <c r="H65" s="10">
+        <v>58.5</v>
+      </c>
+      <c r="I65" s="16">
+        <v>0.14799999999999999</v>
       </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" s="36" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B66" s="25" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C66" s="10" t="s">
         <v>71</v>
@@ -11588,68 +11576,54 @@
     </row>
     <row r="67" spans="1:9">
       <c r="A67" s="36" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B67" s="25" t="s">
         <v>149</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D67" s="10">
-        <v>25</v>
+        <v>9.6</v>
       </c>
       <c r="E67" s="10">
-        <v>24</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="F67" s="10">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="G67" s="10">
-        <v>43.5</v>
+        <v>39</v>
       </c>
       <c r="H67" s="10">
-        <v>58.5</v>
+        <v>42.5</v>
       </c>
       <c r="I67" s="16">
-        <v>0.14799999999999999</v>
+        <v>5.5E-2</v>
       </c>
     </row>
     <row r="68" spans="1:9">
       <c r="A68" s="36" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B68" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="C68" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D68" s="10">
-        <v>9.6</v>
-      </c>
-      <c r="E68" s="10">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="F68" s="10">
-        <v>31</v>
-      </c>
-      <c r="G68" s="10">
-        <v>39</v>
-      </c>
-      <c r="H68" s="10">
-        <v>42.5</v>
-      </c>
-      <c r="I68" s="16">
-        <v>5.5E-2</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="C68" s="10"/>
+      <c r="D68" s="10"/>
+      <c r="E68" s="10"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+      <c r="I68" s="16"/>
     </row>
     <row r="69" spans="1:9">
       <c r="A69" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B69" s="25" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="10"/>
@@ -11661,14 +11635,20 @@
     </row>
     <row r="70" spans="1:9">
       <c r="A70" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="B70" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
+        <v>137</v>
+      </c>
+      <c r="B70" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="C70" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D70" s="10">
+        <v>15.2</v>
+      </c>
+      <c r="E70" s="10">
+        <v>14.2</v>
+      </c>
       <c r="F70" s="10"/>
       <c r="G70" s="10"/>
       <c r="H70" s="10"/>
@@ -11676,149 +11656,140 @@
     </row>
     <row r="71" spans="1:9">
       <c r="A71" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B71" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D71" s="10">
-        <v>15.2</v>
-      </c>
-      <c r="E71" s="10">
-        <v>14.2</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="C71" s="10"/>
+      <c r="D71" s="10"/>
+      <c r="E71" s="10"/>
       <c r="F71" s="10"/>
       <c r="G71" s="10"/>
       <c r="H71" s="10"/>
       <c r="I71" s="16"/>
     </row>
     <row r="72" spans="1:9">
-      <c r="A72" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="B72" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
-      <c r="I72" s="16"/>
+      <c r="A72" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B72" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D72" s="10">
+        <v>17.079999999999998</v>
+      </c>
+      <c r="E72" s="10">
+        <v>16.5</v>
+      </c>
+      <c r="F72" s="10">
+        <v>37</v>
+      </c>
+      <c r="G72" s="10">
+        <v>17.5</v>
+      </c>
+      <c r="H72" s="10">
+        <v>43.5</v>
+      </c>
+      <c r="I72" s="16">
+        <v>2.816625E-2</v>
+      </c>
     </row>
     <row r="73" spans="1:9">
-      <c r="A73" s="17" t="s">
-        <v>146</v>
+      <c r="A73" s="36" t="s">
+        <v>133</v>
       </c>
       <c r="B73" s="25" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="D73" s="10">
-        <v>17.079999999999998</v>
+        <v>18.86</v>
       </c>
       <c r="E73" s="10">
-        <v>16.5</v>
-      </c>
-      <c r="F73" s="10">
-        <v>37</v>
-      </c>
-      <c r="G73" s="10">
-        <v>17.5</v>
-      </c>
-      <c r="H73" s="10">
-        <v>43.5</v>
-      </c>
-      <c r="I73" s="16">
-        <v>2.816625E-2</v>
-      </c>
+        <v>17.239999999999998</v>
+      </c>
+      <c r="F73" s="10"/>
+      <c r="G73" s="10"/>
+      <c r="H73" s="10"/>
+      <c r="I73" s="16"/>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="B74" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="B74" s="25" t="s">
-        <v>137</v>
-      </c>
       <c r="C74" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D74" s="10">
-        <v>18.86</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="E74" s="10">
-        <v>17.239999999999998</v>
-      </c>
-      <c r="F74" s="10"/>
-      <c r="G74" s="10"/>
-      <c r="H74" s="10"/>
-      <c r="I74" s="16"/>
+        <v>16.600000000000001</v>
+      </c>
+      <c r="F74" s="10">
+        <v>40.5</v>
+      </c>
+      <c r="G74" s="10">
+        <v>33.5</v>
+      </c>
+      <c r="H74" s="10">
+        <v>30</v>
+      </c>
+      <c r="I74" s="16">
+        <v>0.41</v>
+      </c>
     </row>
-    <row r="75" spans="1:9">
-      <c r="A75" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="B75" s="25" t="s">
-        <v>139</v>
+    <row r="75" spans="1:9" ht="29">
+      <c r="A75" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B75" s="17" t="s">
+        <v>131</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="D75" s="10">
-        <v>17.600000000000001</v>
+        <v>28.5</v>
       </c>
       <c r="E75" s="10">
-        <v>16.600000000000001</v>
+        <v>27</v>
       </c>
       <c r="F75" s="10">
-        <v>40.5</v>
+        <v>80</v>
       </c>
       <c r="G75" s="10">
-        <v>33.5</v>
+        <v>31.5</v>
       </c>
       <c r="H75" s="10">
-        <v>30</v>
+        <v>53.5</v>
       </c>
       <c r="I75" s="16">
-        <v>0.41</v>
+        <v>0.13500000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="29">
-      <c r="A76" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="B76" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="C76" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D76" s="10">
-        <v>28.5</v>
-      </c>
-      <c r="E76" s="10">
-        <v>27</v>
-      </c>
-      <c r="F76" s="10">
-        <v>80</v>
-      </c>
-      <c r="G76" s="10">
-        <v>31.5</v>
-      </c>
-      <c r="H76" s="10">
-        <v>53.5</v>
-      </c>
-      <c r="I76" s="16">
-        <v>0.13500000000000001</v>
-      </c>
+    <row r="76" spans="1:9">
+      <c r="C76" s="10"/>
+      <c r="D76" s="10"/>
+      <c r="E76" s="10"/>
+      <c r="F76" s="10"/>
+      <c r="G76" s="10"/>
+      <c r="H76" s="10"/>
+      <c r="I76" s="16"/>
     </row>
-    <row r="77" spans="1:9">
+    <row r="77" spans="1:9" ht="23.5">
+      <c r="A77" s="34" t="s">
+        <v>78</v>
+      </c>
       <c r="C77" s="10"/>
       <c r="D77" s="10"/>
       <c r="E77" s="10"/>
@@ -11827,246 +11798,234 @@
       <c r="H77" s="10"/>
       <c r="I77" s="16"/>
     </row>
-    <row r="78" spans="1:9" ht="23.5">
-      <c r="A78" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="C78" s="10"/>
-      <c r="D78" s="10"/>
-      <c r="E78" s="10"/>
-      <c r="F78" s="10"/>
-      <c r="G78" s="10"/>
-      <c r="H78" s="10"/>
-      <c r="I78" s="16"/>
+    <row r="78" spans="1:9">
+      <c r="A78" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F78" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G78" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H78" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I78" s="16" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="79" spans="1:9">
-      <c r="A79" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B79" s="6" t="s">
-        <v>1</v>
+    <row r="79" spans="1:9" s="4" customFormat="1">
+      <c r="A79" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B79" s="21" t="s">
+        <v>164</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F79" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="G79" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I79" s="16" t="s">
-        <v>7</v>
+        <v>40</v>
+      </c>
+      <c r="D79" s="10">
+        <v>11.8</v>
+      </c>
+      <c r="E79" s="10">
+        <v>11.6</v>
+      </c>
+      <c r="F79" s="10">
+        <v>28.4</v>
+      </c>
+      <c r="G79" s="10">
+        <v>31.6</v>
+      </c>
+      <c r="H79" s="10">
+        <v>30</v>
+      </c>
+      <c r="I79" s="16">
+        <v>2.7E-2</v>
       </c>
     </row>
     <row r="80" spans="1:9" s="4" customFormat="1">
-      <c r="A80" s="17" t="s">
-        <v>156</v>
+      <c r="A80" s="15" t="s">
+        <v>154</v>
       </c>
       <c r="B80" s="21" t="s">
-        <v>168</v>
+        <v>100</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D80" s="10">
-        <v>11.8</v>
+        <v>12.75</v>
       </c>
       <c r="E80" s="10">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="F80" s="10">
-        <v>28.4</v>
+        <v>37.5</v>
       </c>
       <c r="G80" s="10">
-        <v>31.6</v>
+        <v>28.2</v>
       </c>
       <c r="H80" s="10">
-        <v>30</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I80" s="16">
-        <v>2.7E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="81" spans="1:9" s="4" customFormat="1">
       <c r="A81" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="B81" s="21" t="s">
-        <v>100</v>
+        <v>75</v>
+      </c>
+      <c r="B81" s="17" t="s">
+        <v>155</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="D81" s="10">
-        <v>12.75</v>
+        <v>12</v>
       </c>
       <c r="E81" s="10">
-        <v>11.2</v>
+        <v>11.23</v>
       </c>
       <c r="F81" s="10">
-        <v>37.5</v>
+        <v>36</v>
       </c>
       <c r="G81" s="10">
-        <v>28.2</v>
+        <v>27</v>
       </c>
       <c r="H81" s="10">
-        <v>34.799999999999997</v>
+        <v>27</v>
       </c>
       <c r="I81" s="16">
-        <v>3.6999999999999998E-2</v>
+        <v>2.6244E-2</v>
       </c>
     </row>
     <row r="82" spans="1:9" s="4" customFormat="1">
       <c r="A82" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B82" s="17" t="s">
-        <v>158</v>
+        <v>76</v>
+      </c>
+      <c r="B82" s="21" t="s">
+        <v>106</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="D82" s="10">
-        <v>12</v>
+        <v>12.75</v>
       </c>
       <c r="E82" s="10">
-        <v>11.23</v>
+        <v>11.2</v>
       </c>
       <c r="F82" s="10">
-        <v>36</v>
+        <v>37.5</v>
       </c>
       <c r="G82" s="10">
-        <v>27</v>
+        <v>28.2</v>
       </c>
       <c r="H82" s="10">
-        <v>27</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I82" s="16">
-        <v>2.6244E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="83" spans="1:9" s="4" customFormat="1">
       <c r="A83" s="15" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="B83" s="21" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D83" s="10">
-        <v>12.75</v>
+        <v>11</v>
       </c>
       <c r="E83" s="10">
-        <v>11.2</v>
+        <v>13</v>
       </c>
       <c r="F83" s="10">
-        <v>37.5</v>
+        <v>35</v>
       </c>
       <c r="G83" s="10">
-        <v>28.2</v>
+        <v>22</v>
       </c>
       <c r="H83" s="10">
-        <v>34.799999999999997</v>
+        <v>39</v>
       </c>
       <c r="I83" s="16">
-        <v>3.6999999999999998E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="84" spans="1:9" s="4" customFormat="1">
       <c r="A84" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B84" s="21" t="s">
-        <v>169</v>
+        <v>150</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>166</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="D84" s="10">
-        <v>11</v>
+        <v>9.5440000000000005</v>
       </c>
       <c r="E84" s="10">
-        <v>13</v>
+        <v>8.5440000000000005</v>
       </c>
       <c r="F84" s="10">
-        <v>35</v>
+        <v>44.8</v>
       </c>
       <c r="G84" s="10">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H84" s="10">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I84" s="16">
-        <v>0.03</v>
+        <v>1.2999999999999999E-2</v>
       </c>
     </row>
     <row r="85" spans="1:9" s="4" customFormat="1">
       <c r="A85" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="B85" s="17" t="s">
-        <v>170</v>
+        <v>151</v>
+      </c>
+      <c r="B85" s="22" t="s">
+        <v>152</v>
       </c>
       <c r="C85" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D85" s="10">
-        <v>9.5440000000000005</v>
-      </c>
-      <c r="E85" s="10">
-        <v>8.5440000000000005</v>
-      </c>
-      <c r="F85" s="10">
-        <v>44.8</v>
-      </c>
-      <c r="G85" s="10">
-        <v>30</v>
-      </c>
-      <c r="H85" s="10">
-        <v>10</v>
-      </c>
-      <c r="I85" s="16">
-        <v>1.2999999999999999E-2</v>
-      </c>
+      <c r="D85" s="10"/>
+      <c r="E85" s="10"/>
+      <c r="F85" s="10"/>
+      <c r="G85" s="10"/>
+      <c r="H85" s="10"/>
+      <c r="I85" s="16"/>
     </row>
-    <row r="86" spans="1:9" s="4" customFormat="1">
-      <c r="A86" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="B86" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="C86" s="10" t="s">
-        <v>70</v>
-      </c>
+    <row r="86" spans="1:9">
+      <c r="C86" s="10"/>
       <c r="D86" s="10"/>
       <c r="E86" s="10"/>
       <c r="F86" s="10"/>
       <c r="G86" s="10"/>
       <c r="H86" s="10"/>
       <c r="I86" s="16"/>
-    </row>
-    <row r="87" spans="1:9">
-      <c r="C87" s="10"/>
-      <c r="D87" s="10"/>
-      <c r="E87" s="10"/>
-      <c r="F87" s="10"/>
-      <c r="G87" s="10"/>
-      <c r="H87" s="10"/>
-      <c r="I87" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="30" type="noConversion"/>

</xml_diff>